<commit_message>
push latest update He-Xe exp
</commit_message>
<xml_diff>
--- a/input/input_exp_He-Xe-T20-P725.xlsx
+++ b/input/input_exp_He-Xe-T20-P725.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pennstateoffice365-my.sharepoint.com/personal/izg5132_psu_edu/Documents/06_PHD_EME_PSU/00 RESEARCH/PHD UHS PROJECT/MATLAB-GITHUB/UHS-CF-Dispersion-Exps2/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="833" documentId="11_F25DC773A252ABDACC1048B8D1997AFC5ADE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{48AC9912-8F9D-470D-AF38-6F86DFF3F6F9}"/>
+  <xr:revisionPtr revIDLastSave="845" documentId="11_F25DC773A252ABDACC1048B8D1997AFC5ADE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{54EAA9D5-C006-4920-85A2-C48E8597344C}"/>
   <bookViews>
-    <workbookView xWindow="1152" yWindow="1152" windowWidth="17280" windowHeight="8928" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="64">
   <si>
     <t>path</t>
   </si>
@@ -225,6 +225,9 @@
   </si>
   <si>
     <t>CF</t>
+  </si>
+  <si>
+    <t>1A</t>
   </si>
 </sst>
 </file>
@@ -569,29 +572,29 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AI4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30.44140625" customWidth="1"/>
-    <col min="2" max="2" width="9.88671875" style="4" customWidth="1"/>
-    <col min="3" max="3" width="7.6640625" style="4" customWidth="1"/>
-    <col min="4" max="7" width="7.33203125" customWidth="1"/>
-    <col min="8" max="10" width="7.109375" customWidth="1"/>
-    <col min="11" max="11" width="7.33203125" customWidth="1"/>
-    <col min="12" max="16" width="10.109375" customWidth="1"/>
-    <col min="17" max="21" width="12.88671875" customWidth="1"/>
-    <col min="22" max="25" width="30.33203125" customWidth="1"/>
-    <col min="26" max="26" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.42578125" customWidth="1"/>
+    <col min="2" max="2" width="9.85546875" style="4" customWidth="1"/>
+    <col min="3" max="3" width="7.7109375" style="4" customWidth="1"/>
+    <col min="4" max="7" width="7.28515625" customWidth="1"/>
+    <col min="8" max="10" width="7.140625" customWidth="1"/>
+    <col min="11" max="11" width="7.28515625" customWidth="1"/>
+    <col min="12" max="16" width="10.140625" customWidth="1"/>
+    <col min="17" max="21" width="12.85546875" customWidth="1"/>
+    <col min="22" max="25" width="30.28515625" customWidth="1"/>
+    <col min="26" max="26" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="16" customWidth="1"/>
-    <col min="29" max="29" width="35.33203125" style="1" customWidth="1"/>
-    <col min="30" max="30" width="21.109375" style="1" customWidth="1"/>
-    <col min="31" max="31" width="21.33203125" style="1" customWidth="1"/>
+    <col min="29" max="29" width="35.28515625" style="1" customWidth="1"/>
+    <col min="30" max="30" width="21.140625" style="1" customWidth="1"/>
+    <col min="31" max="31" width="21.28515625" style="1" customWidth="1"/>
     <col min="32" max="32" width="26" style="1" customWidth="1"/>
-    <col min="33" max="33" width="18.33203125" style="2" customWidth="1"/>
-    <col min="34" max="34" width="20.33203125" style="2" customWidth="1"/>
-    <col min="35" max="35" width="11.6640625" customWidth="1"/>
+    <col min="33" max="33" width="18.28515625" style="2" customWidth="1"/>
+    <col min="34" max="34" width="20.28515625" style="2" customWidth="1"/>
+    <col min="35" max="35" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>21</v>
       </c>
@@ -698,7 +701,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:35" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:35" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="4" t="s">
         <v>15</v>
       </c>
@@ -754,7 +757,7 @@
       <c r="AG2" s="1"/>
       <c r="AH2" s="1"/>
     </row>
-    <row r="3" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:35" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>50</v>
       </c>
@@ -810,13 +813,13 @@
         <v>0.29399999999999998</v>
       </c>
       <c r="S3">
-        <v>30.9</v>
+        <v>35.4</v>
       </c>
       <c r="T3">
-        <v>13.1</v>
+        <v>26.1</v>
       </c>
       <c r="U3">
-        <v>103.8</v>
+        <v>121.3</v>
       </c>
       <c r="V3" t="s">
         <v>46</v>
@@ -827,8 +830,8 @@
       <c r="X3">
         <v>2</v>
       </c>
-      <c r="Y3">
-        <v>1</v>
+      <c r="Y3" t="s">
+        <v>63</v>
       </c>
       <c r="Z3" s="3">
         <v>46010.450706018521</v>
@@ -855,7 +858,7 @@
       <c r="AH3" s="6"/>
       <c r="AI3" s="1"/>
     </row>
-    <row r="4" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:35" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>51</v>
       </c>
@@ -911,13 +914,13 @@
         <v>0.29399999999999998</v>
       </c>
       <c r="S4">
-        <v>30.9</v>
+        <v>35.4</v>
       </c>
       <c r="T4">
-        <v>13.1</v>
+        <v>26.1</v>
       </c>
       <c r="U4">
-        <v>103.8</v>
+        <v>121.3</v>
       </c>
       <c r="V4" t="s">
         <v>46</v>
@@ -928,8 +931,8 @@
       <c r="X4">
         <v>2</v>
       </c>
-      <c r="Y4">
-        <v>1</v>
+      <c r="Y4" t="s">
+        <v>63</v>
       </c>
       <c r="Z4" s="3">
         <v>46007.657638888886</v>

</xml_diff>